<commit_message>
Add real URLs to all 99 source links across xlsx and index.html
Fixed 65 mismatched/missing hyperlinks in the xlsx (URLs were
scrambled across wrong cells). Added real href URLs to all 99
public source links in index.html (previously all href="#").
Only 9 internal/Charles Acknin sources remain without URLs.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/Skyways_Timeline_Data.xlsx
+++ b/Data/Skyways_Timeline_Data.xlsx
@@ -150,7 +150,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -262,6 +262,15 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1368,12 +1377,12 @@
           <t>Product</t>
         </is>
       </c>
-      <c r="G14" s="18" t="inlineStr">
+      <c r="G14" s="39" t="inlineStr">
         <is>
           <t>The Drone Girl — Inside Skyways</t>
         </is>
       </c>
-      <c r="H14" s="18" t="inlineStr">
+      <c r="H14" s="39" t="inlineStr">
         <is>
           <t>SBIR.gov — V2.5 referenced</t>
         </is>
@@ -1423,17 +1432,17 @@
           <t>Defense — U.S. Navy</t>
         </is>
       </c>
-      <c r="G15" s="11" t="inlineStr">
+      <c r="G15" s="40" t="inlineStr">
         <is>
           <t>The War Zone — Navy Tests Autonomous Supply Drone From Supercarrier</t>
         </is>
       </c>
-      <c r="H15" s="11" t="inlineStr">
+      <c r="H15" s="40" t="inlineStr">
         <is>
           <t>USNI News — Navy Considering Drone Delivery (Aug 2021)</t>
         </is>
       </c>
-      <c r="I15" s="11" t="inlineStr">
+      <c r="I15" s="40" t="inlineStr">
         <is>
           <t>Maritime Executive — Carrier USS Ford Tests Air Cargo Drone</t>
         </is>
@@ -1482,7 +1491,7 @@
           <t>Contract — U.S. Air Force</t>
         </is>
       </c>
-      <c r="G16" s="16" t="inlineStr">
+      <c r="G16" s="37" t="inlineStr">
         <is>
           <t>SBIR.gov — Award FA8649-21-P-0539</t>
         </is>
@@ -1533,12 +1542,12 @@
           <t>Contract — Commercial</t>
         </is>
       </c>
-      <c r="G17" s="16" t="inlineStr">
+      <c r="G17" s="37" t="inlineStr">
         <is>
           <t>SBIR.gov — Phase I references O&amp;G</t>
         </is>
       </c>
-      <c r="H17" s="16" t="inlineStr">
+      <c r="H17" s="37" t="inlineStr">
         <is>
           <t>The Drone Girl — Inside Skyways</t>
         </is>
@@ -1588,7 +1597,7 @@
           <t>Defense</t>
         </is>
       </c>
-      <c r="G18" s="11" t="inlineStr">
+      <c r="G18" s="40" t="inlineStr">
         <is>
           <t>USNI News — Navy Considering Drone Delivery (Aug 2021)</t>
         </is>
@@ -1700,7 +1709,7 @@
           <t>Contract — U.S. Air Force</t>
         </is>
       </c>
-      <c r="G20" s="16" t="inlineStr">
+      <c r="G20" s="37" t="inlineStr">
         <is>
           <t>SBIR.gov — Skyways Portfolio</t>
         </is>
@@ -1756,17 +1765,17 @@
           <t>Defense</t>
         </is>
       </c>
-      <c r="G21" s="11" t="inlineStr">
+      <c r="G21" s="40" t="inlineStr">
         <is>
           <t>NAVAIR — Navy Demonstrates Unmanned Cargo Delivery (Dec 2022)</t>
         </is>
       </c>
-      <c r="H21" s="11" t="inlineStr">
+      <c r="H21" s="40" t="inlineStr">
         <is>
           <t>USNI News — Navy to Deploy Four Cargo Drones on Carrier (Apr 2022)</t>
         </is>
       </c>
-      <c r="I21" s="11" t="inlineStr">
+      <c r="I21" s="40" t="inlineStr">
         <is>
           <t>DroneXL — Navy Drone Delivery Trials (Jan 2023)</t>
         </is>
@@ -1871,22 +1880,22 @@
           <t>Defense — U.S. Navy / USMC</t>
         </is>
       </c>
-      <c r="G23" s="11" t="inlineStr">
+      <c r="G23" s="40" t="inlineStr">
         <is>
           <t>DVIDS — NAWCAD Teams with MSC, Marines (Jun 2023)</t>
         </is>
       </c>
-      <c r="H23" s="11" t="inlineStr">
+      <c r="H23" s="40" t="inlineStr">
         <is>
           <t>MSC/Navy.mil — NAWCAD Teams with MSC, Marines (Jun 2023)</t>
         </is>
       </c>
-      <c r="I23" s="11" t="inlineStr">
+      <c r="I23" s="40" t="inlineStr">
         <is>
           <t>Inside Unmanned Systems — Navy Drone Delivery at Sea</t>
         </is>
       </c>
-      <c r="J23" s="0" t="inlineStr">
+      <c r="J23" s="38" t="inlineStr">
         <is>
           <t>Navy.mil — Fleet Battle Problem 23-1</t>
         </is>
@@ -1935,7 +1944,7 @@
           <t>Product</t>
         </is>
       </c>
-      <c r="G24" s="18" t="inlineStr">
+      <c r="G24" s="39" t="inlineStr">
         <is>
           <t>sUAS News — Skyways V3</t>
         </is>
@@ -1986,32 +1995,32 @@
           <t>Defense</t>
         </is>
       </c>
-      <c r="G25" s="11" t="inlineStr">
+      <c r="G25" s="40" t="inlineStr">
         <is>
           <t>Defense News — Navy tests drones for medical supply at RIMPAC (Jul 2024)</t>
         </is>
       </c>
-      <c r="H25" s="11" t="inlineStr">
+      <c r="H25" s="40" t="inlineStr">
         <is>
           <t>The Aviationist — U.S. Navy Tests VTOL Drones for Cargo (Jul 2024)</t>
         </is>
       </c>
-      <c r="I25" s="11" t="inlineStr">
+      <c r="I25" s="40" t="inlineStr">
         <is>
           <t>Eurasian Times — US Navy Demonstrates Unmanned Cargo Delivery</t>
         </is>
       </c>
-      <c r="J25" s="0" t="inlineStr">
+      <c r="J25" s="38" t="inlineStr">
         <is>
           <t>SURFPAC/Navy.mil — USS Curtis Wilbur Tests Drones During RIMPAC Trident Warrior 2024</t>
         </is>
       </c>
-      <c r="K25" s="11" t="inlineStr">
+      <c r="K25" s="40" t="inlineStr">
         <is>
           <t>Battle Updates — Unmanned Systems Update</t>
         </is>
       </c>
-      <c r="L25" s="10" t="inlineStr">
+      <c r="L25" s="40" t="inlineStr">
         <is>
           <t>DVIDS — USS Curtis Wilbur Tests Drones During RIMPAC Trident Warrior 2024</t>
         </is>
@@ -2114,7 +2123,7 @@
           <t>Contract — U.S. Air Force</t>
         </is>
       </c>
-      <c r="G27" s="16" t="inlineStr">
+      <c r="G27" s="37" t="inlineStr">
         <is>
           <t>SBIR.gov — Skyways Portfolio (Fact Error: Listed $3.55M STRATFI amount; Charles says figure is wrong and timeline differs)</t>
         </is>
@@ -2322,17 +2331,17 @@
           <t>Funding</t>
         </is>
       </c>
-      <c r="G30" s="16" t="inlineStr">
+      <c r="G30" s="37" t="inlineStr">
         <is>
           <t>Business Wire — $5M Debt Facility Announcement (Fact Error: Reported $5M debt facility only; total private raise was ~$7M for STRATFI 1:1:2 matching)</t>
         </is>
       </c>
-      <c r="H30" s="16" t="inlineStr">
+      <c r="H30" s="37" t="inlineStr">
         <is>
           <t>DroneLife — Skyways Secures $5M for Production (Jul 2025)</t>
         </is>
       </c>
-      <c r="I30" s="16" t="inlineStr">
+      <c r="I30" s="37" t="inlineStr">
         <is>
           <t>Skyways Newsroom</t>
         </is>
@@ -2386,17 +2395,17 @@
           <t>Defense — DoD</t>
         </is>
       </c>
-      <c r="G31" s="11" t="inlineStr">
+      <c r="G31" s="40" t="inlineStr">
         <is>
           <t>KX News — Project ULTRA expands, $100M ceiling (Jul 2025)</t>
         </is>
       </c>
-      <c r="H31" s="11" t="inlineStr">
+      <c r="H31" s="40" t="inlineStr">
         <is>
           <t>Air Cargo Week — Skyways completes historic flights (Aug 2025)</t>
         </is>
       </c>
-      <c r="I31" s="11" t="inlineStr">
+      <c r="I31" s="40" t="inlineStr">
         <is>
           <t>DroneLife — Skyways Historic Cargo Drone Flights (Aug 2025)</t>
         </is>
@@ -2406,12 +2415,12 @@
           <t>Charles Acknin Source Correction — Sponsored by OUSD (not USD(A&amp;S)); flights were BVLOS in the NAS</t>
         </is>
       </c>
-      <c r="K31" s="11" t="inlineStr">
+      <c r="K31" s="40" t="inlineStr">
         <is>
           <t>Business Wire — Project ULTRA Press Release (Fact Error: Listed sponsor as USD(A&amp;S); correct sponsor is OUSD; did not specify flights were BVLOS in NAS)</t>
         </is>
       </c>
-      <c r="L31" s="11" t="inlineStr">
+      <c r="L31" s="40" t="inlineStr">
         <is>
           <t>Skyways Newsroom (Fact Error: Listed sponsor as USD(A&amp;S); correct sponsor is OUSD; did not specify flights were BVLOS in NAS)</t>
         </is>
@@ -2458,27 +2467,27 @@
           <t>Product</t>
         </is>
       </c>
-      <c r="G32" s="18" t="inlineStr">
+      <c r="G32" s="39" t="inlineStr">
         <is>
           <t>DroneLife — Skyways Historic Cargo Drone Flights (Aug 2025)</t>
         </is>
       </c>
-      <c r="H32" s="18" t="inlineStr">
+      <c r="H32" s="39" t="inlineStr">
         <is>
           <t>DroneXL — Skyways Autonomous Drone Fleet (Feb 2026)</t>
         </is>
       </c>
-      <c r="I32" s="18" t="inlineStr">
+      <c r="I32" s="39" t="inlineStr">
         <is>
           <t>Skyways Newsroom</t>
         </is>
       </c>
-      <c r="J32" s="0" t="inlineStr">
+      <c r="J32" s="38" t="inlineStr">
         <is>
           <t>The Drone Girl — Inside Skyways (Nov 2025)</t>
         </is>
       </c>
-      <c r="K32" s="8" t="inlineStr">
+      <c r="K32" s="39" t="inlineStr">
         <is>
           <t>The Drone Girl — From Cargo to Commuters Roadmap (Dec 2025)</t>
         </is>
@@ -2530,12 +2539,12 @@
           <t>Product</t>
         </is>
       </c>
-      <c r="G33" s="18" t="inlineStr">
+      <c r="G33" s="39" t="inlineStr">
         <is>
           <t>DroneXL — Skyways Autonomous Drone Fleet (Feb 2026)</t>
         </is>
       </c>
-      <c r="H33" s="18" t="inlineStr">
+      <c r="H33" s="39" t="inlineStr">
         <is>
           <t>The Drone Girl — Inside Skyways (Nov 2025)</t>
         </is>
@@ -2589,7 +2598,7 @@
           <t>Milestone</t>
         </is>
       </c>
-      <c r="G34" s="21" t="inlineStr">
+      <c r="G34" s="38" t="inlineStr">
         <is>
           <t>The Drone Girl — Inside Skyways (Nov 2025)</t>
         </is>
@@ -2599,7 +2608,7 @@
           <t>DroneXL — Skyways Autonomous Drone Fleet (Feb 2026)</t>
         </is>
       </c>
-      <c r="I34" s="21" t="inlineStr">
+      <c r="I34" s="38" t="inlineStr">
         <is>
           <t>Energy Global — RWE pioneers cargo drone ops (Oct 2025)</t>
         </is>
@@ -2609,7 +2618,7 @@
           <t>Charles Acknin Source Correction — First international aircraft deliveries: Skyports ~Feb 2025, ANA ~Apr 2025</t>
         </is>
       </c>
-      <c r="K34" s="21" t="inlineStr">
+      <c r="K34" s="38" t="inlineStr">
         <is>
           <t>GlobeNewswire — Skyways Historic Cargo Deliveries</t>
         </is>
@@ -2657,27 +2666,27 @@
           <t>Contract — RWE (Germany)</t>
         </is>
       </c>
-      <c r="G35" s="16" t="inlineStr">
+      <c r="G35" s="37" t="inlineStr">
         <is>
           <t>RWE — Pioneers cargo drone operations (Oct 2025)</t>
         </is>
       </c>
-      <c r="H35" s="16" t="inlineStr">
+      <c r="H35" s="37" t="inlineStr">
         <is>
           <t>Unmanned Systems Technology — Autonomous Cargo Drone (Oct 2025)</t>
         </is>
       </c>
-      <c r="I35" s="16" t="inlineStr">
+      <c r="I35" s="37" t="inlineStr">
         <is>
           <t>eVTOL Insights — Germany first long-range deliveries (Oct 2025)</t>
         </is>
       </c>
-      <c r="J35" s="0" t="inlineStr">
+      <c r="J35" s="38" t="inlineStr">
         <is>
           <t>DroneXL — Skyways Drone Cuts Supply Time (Oct 2025)</t>
         </is>
       </c>
-      <c r="K35" s="16" t="inlineStr">
+      <c r="K35" s="37" t="inlineStr">
         <is>
           <t>DroneLife — Germany First Long-Range Deliveries (Oct 2025)</t>
         </is>
@@ -2725,17 +2734,17 @@
           <t>Contract — ANA Holdings (Japan)</t>
         </is>
       </c>
-      <c r="G36" s="16" t="inlineStr">
+      <c r="G36" s="37" t="inlineStr">
         <is>
           <t>Yomiuri Shimbun — ANA builds drone logistics network (Jan 2026)</t>
         </is>
       </c>
-      <c r="H36" s="16" t="inlineStr">
+      <c r="H36" s="37" t="inlineStr">
         <is>
           <t>Japan Today / Kyodo — ANA drone delivery by FY2028</t>
         </is>
       </c>
-      <c r="I36" s="16" t="inlineStr">
+      <c r="I36" s="37" t="inlineStr">
         <is>
           <t>Payload Asia — ANA Okinawa medical drone trials (Mar 2026)</t>
         </is>
@@ -2745,12 +2754,12 @@
           <t>Charles Acknin Source Correction — Coordinate messaging with Jessica Hogan; ANA cautious about public disclosure due to DoD ties</t>
         </is>
       </c>
-      <c r="K36" s="16" t="inlineStr">
+      <c r="K36" s="37" t="inlineStr">
         <is>
           <t>The Drone Girl — Inside Skyways (Nov 2025)</t>
         </is>
       </c>
-      <c r="L36" s="16" t="inlineStr">
+      <c r="L36" s="37" t="inlineStr">
         <is>
           <t>The Drone Girl — From cargo to commuters (Dec 2025)</t>
         </is>
@@ -2797,17 +2806,17 @@
           <t>Milestone</t>
         </is>
       </c>
-      <c r="G37" s="14" t="inlineStr">
+      <c r="G37" s="41" t="inlineStr">
         <is>
           <t>The Drone Girl — Inside Skyways aspirations (Nov 2025)</t>
         </is>
       </c>
-      <c r="H37" s="14" t="inlineStr">
+      <c r="H37" s="41" t="inlineStr">
         <is>
           <t>The Drone Girl — From cargo to commuters roadmap (Dec 2025)</t>
         </is>
       </c>
-      <c r="I37" s="14" t="inlineStr">
+      <c r="I37" s="41" t="inlineStr">
         <is>
           <t>KXAN Austin/NBC — Austin aviation company scaling drones (Nov 2025)</t>
         </is>
@@ -2856,17 +2865,17 @@
           <t>Milestone</t>
         </is>
       </c>
-      <c r="G38" s="14" t="inlineStr">
+      <c r="G38" s="41" t="inlineStr">
         <is>
           <t>Austin American-Statesman — In-depth Skyways profile (Feb 2026) (Fact Error: Reported approximately 30 employees; company finished 2025 at ~39 employees per Charles)</t>
         </is>
       </c>
-      <c r="H38" s="14" t="inlineStr">
+      <c r="H38" s="41" t="inlineStr">
         <is>
           <t>DroneXL — Skyways Plans Worlds Largest Fleet (Feb 2026)</t>
         </is>
       </c>
-      <c r="I38" s="14" t="inlineStr">
+      <c r="I38" s="41" t="inlineStr">
         <is>
           <t>GlobeNewswire — Skyways Strengthens Leadership (Jan 2026)</t>
         </is>
@@ -2920,12 +2929,12 @@
           <t>Milestone</t>
         </is>
       </c>
-      <c r="G39" s="14" t="inlineStr">
+      <c r="G39" s="41" t="inlineStr">
         <is>
           <t>Payload Asia — ANA completes Okinawa trials (Mar 2026)</t>
         </is>
       </c>
-      <c r="H39" s="14" t="inlineStr">
+      <c r="H39" s="41" t="inlineStr">
         <is>
           <t>Japan Today — ANA drone delivery by FY2028</t>
         </is>
@@ -2975,12 +2984,12 @@
           <t>Upcoming</t>
         </is>
       </c>
-      <c r="G40" s="18" t="inlineStr">
+      <c r="G40" s="39" t="inlineStr">
         <is>
           <t>DroneXL — Skyways Autonomous Drone Fleet (Feb 2026)</t>
         </is>
       </c>
-      <c r="H40" s="18" t="inlineStr">
+      <c r="H40" s="39" t="inlineStr">
         <is>
           <t>ADrones — Skyways Plans Largest Fleet (Feb 2026)</t>
         </is>
@@ -3030,12 +3039,12 @@
           <t>Upcoming</t>
         </is>
       </c>
-      <c r="G41" s="18" t="inlineStr">
+      <c r="G41" s="39" t="inlineStr">
         <is>
           <t>DroneXL — Skyways Autonomous Drone Fleet (Feb 2026)</t>
         </is>
       </c>
-      <c r="H41" s="18" t="inlineStr">
+      <c r="H41" s="39" t="inlineStr">
         <is>
           <t>ADrones — Skyways Plans Largest Fleet (Feb 2026)</t>
         </is>
@@ -4044,60 +4053,89 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K29" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N29" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P29" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K31" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K32" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K29" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N29" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P29" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K31" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J32" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K32" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J35" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId107"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>